<commit_message>
Update Test Case All-Uses Coverage
</commit_message>
<xml_diff>
--- a/table/Test Case Sheet.xlsx
+++ b/table/Test Case Sheet.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\c\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GymFeeCalculator\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CBE1EEA-15AA-4AB3-8909-B912BE244E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E05D31-DB3E-4F0D-822E-ADCA8FA7BAF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12216" activeTab="2" xr2:uid="{BB4CBC31-628A-4A18-86E6-6709F765FC93}"/>
+    <workbookView xWindow="24" yWindow="384" windowWidth="23016" windowHeight="12216" activeTab="3" xr2:uid="{BB4CBC31-628A-4A18-86E6-6709F765FC93}"/>
   </bookViews>
   <sheets>
     <sheet name="Kiểm thử biên" sheetId="1" r:id="rId1"/>
     <sheet name="Kiểm thử bảng quyết định" sheetId="2" r:id="rId2"/>
     <sheet name="Kiểm thử C2" sheetId="3" r:id="rId3"/>
+    <sheet name="Kiểm thử All-Uses Coverage" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="218">
   <si>
     <t>TC01</t>
   </si>
@@ -545,6 +546,153 @@
   </si>
   <si>
     <t>TEST CASE CỤ THỂ</t>
+  </si>
+  <si>
+    <t>(1, 6, 22, 1)</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2F → 3F → 4F → 5 → 6 → 7 → 8 → 9 → 10</t>
+  </si>
+  <si>
+    <t>9 → 10</t>
+  </si>
+  <si>
+    <t>(phiThuc, 9→10) c-use</t>
+  </si>
+  <si>
+    <t>8 → 9</t>
+  </si>
+  <si>
+    <t>(giamSV, 8→9) c-use</t>
+  </si>
+  <si>
+    <t>(1, 6, 56, 0)</t>
+  </si>
+  <si>
+    <t>7 → 8 → 9</t>
+  </si>
+  <si>
+    <t>(giamTuoi, 7→9) c-use</t>
+  </si>
+  <si>
+    <t>(1, 6, 30, 0)</t>
+  </si>
+  <si>
+    <t>6 → 7 → 8 → 9</t>
+  </si>
+  <si>
+    <t>(heSoThang, 6→9) c-use</t>
+  </si>
+  <si>
+    <t>5 → 6 → 7 → 8 → 9</t>
+  </si>
+  <si>
+    <t>(giaGoc, 5→9) c-use</t>
+  </si>
+  <si>
+    <t>(3, 1, 40, 0)</t>
+  </si>
+  <si>
+    <t>5 → 5</t>
+  </si>
+  <si>
+    <t>(donGia, 5→5) c-use</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2F → 3F → 4F → 5 → 6 → 7 → 8</t>
+  </si>
+  <si>
+    <t>(coSV, 0→8) c-use</t>
+  </si>
+  <si>
+    <t>(2, 6, 16, 0)</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2F → 3F → 4F → 5 → 6 → 7</t>
+  </si>
+  <si>
+    <t>(doTuoi, 0→7) c-use</t>
+  </si>
+  <si>
+    <t>(2, 4, 30, 0)</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2F → 3F → 4F → 5 → 6</t>
+  </si>
+  <si>
+    <t>(soThang, 0→6) c-use</t>
+  </si>
+  <si>
+    <t>(1, 1, 20, 0)</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2F → 3F → 4F → 5</t>
+  </si>
+  <si>
+    <t>(soThang, 0→5) c-use</t>
+  </si>
+  <si>
+    <t>(loaiGoi, 0→5) c-use</t>
+  </si>
+  <si>
+    <t>(1, 5, 20, 2)</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2F → 3F → 4T → 11</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2F → 3F → 4</t>
+  </si>
+  <si>
+    <t>(coSV, 0→4) p-use</t>
+  </si>
+  <si>
+    <t>(1, 5, 14, 0)</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2F → 3T → 11</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2F → 3</t>
+  </si>
+  <si>
+    <t>(doTuoi, 0→3) p-use</t>
+  </si>
+  <si>
+    <t>(1, 13, 20, 0)</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2T → 11</t>
+  </si>
+  <si>
+    <t>0 → 1F → 2</t>
+  </si>
+  <si>
+    <t>(soThang, 0→2) p-use</t>
+  </si>
+  <si>
+    <t>(4, 5, 20, 0)</t>
+  </si>
+  <si>
+    <t>0 → 1T → 11</t>
+  </si>
+  <si>
+    <t>0 → 1</t>
+  </si>
+  <si>
+    <t>(loaiGoi, 0→1) p-use</t>
+  </si>
+  <si>
+    <t>Test case (loaiGoi, soThang, doTuoi, coSV)</t>
+  </si>
+  <si>
+    <t>Complete path</t>
+  </si>
+  <si>
+    <t>Def-clear path</t>
+  </si>
+  <si>
+    <t>DU-pair</t>
   </si>
 </sst>
 </file>
@@ -647,7 +795,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -661,18 +809,145 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="44">
+  <dxfs count="52">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -690,119 +965,6 @@
         <family val="1"/>
         <scheme val="major"/>
       </font>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -986,6 +1148,114 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <strike val="0"/>
@@ -1004,68 +1274,16 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
         <family val="1"/>
@@ -1272,7 +1490,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -1290,7 +1508,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -1299,115 +1517,190 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
         <family val="1"/>
@@ -1428,73 +1721,88 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D4DFA908-A1A4-4432-A9F0-75BB34DC8BA7}" name="Table3" displayName="Table3" ref="A1:I29" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D4DFA908-A1A4-4432-A9F0-75BB34DC8BA7}" name="Table3" displayName="Table3" ref="A1:I29" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
   <autoFilter ref="A1:I29" xr:uid="{D4DFA908-A1A4-4432-A9F0-75BB34DC8BA7}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{EAF02433-F651-42B5-9F4E-169AF35E6987}" name="TC" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{2E2E6E79-7DB1-479C-9F5A-F587E62EFF72}" name="Biến thay đổi" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{E454FB94-B1EE-42E7-B122-396ED713A4D3}" name="Loại biên" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{70F4EE6B-8123-41AB-8A9B-90AA18B646FF}" name="loaiGoi" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{9FC24758-6ADB-4593-A812-66D3FFC8C6FC}" name="soThang" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{A5913B19-5A4B-4A31-A6EB-FFB56BE30C8C}" name="doTuoi" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{297D8E6B-44BC-4B47-808E-83AE19DFCA45}" name="coSinhVien" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{094DFBF4-96D3-40B7-B4E5-82DFC3AF9F87}" name="Expected Output" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{9B600A2F-5707-4C1E-BEDB-0DA1657FDCA9}" name="Result" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{EAF02433-F651-42B5-9F4E-169AF35E6987}" name="TC" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{2E2E6E79-7DB1-479C-9F5A-F587E62EFF72}" name="Biến thay đổi" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{E454FB94-B1EE-42E7-B122-396ED713A4D3}" name="Loại biên" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{70F4EE6B-8123-41AB-8A9B-90AA18B646FF}" name="loaiGoi" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{9FC24758-6ADB-4593-A812-66D3FFC8C6FC}" name="soThang" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{A5913B19-5A4B-4A31-A6EB-FFB56BE30C8C}" name="doTuoi" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{297D8E6B-44BC-4B47-808E-83AE19DFCA45}" name="coSinhVien" dataDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{094DFBF4-96D3-40B7-B4E5-82DFC3AF9F87}" name="Expected Output" dataDxfId="28"/>
+    <tableColumn id="9" xr3:uid="{9B600A2F-5707-4C1E-BEDB-0DA1657FDCA9}" name="Result" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F844E8AE-F637-4B45-90FB-D0FE93411DE1}" name="Table2" displayName="Table2" ref="A1:R21" totalsRowShown="0" headerRowDxfId="25" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F844E8AE-F637-4B45-90FB-D0FE93411DE1}" name="Table2" displayName="Table2" ref="A1:R21" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A1:R21" xr:uid="{F844E8AE-F637-4B45-90FB-D0FE93411DE1}"/>
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{6DD44F37-B7A8-4D2E-917F-A37F4DB2889D}" name="Column1" dataDxfId="43"/>
+    <tableColumn id="1" xr3:uid="{6DD44F37-B7A8-4D2E-917F-A37F4DB2889D}" name="Column1" dataDxfId="24"/>
     <tableColumn id="2" xr3:uid="{9B6651BA-8E08-4A07-B184-8EE746DDE095}" name="Column2"/>
-    <tableColumn id="3" xr3:uid="{F80A0028-6831-49DC-A737-1843B2BDFB25}" name="Column3" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{B38F8820-4A19-4584-B056-E19957264855}" name="Column4" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{3356337E-64E9-4C20-A5B2-665734CA49EE}" name="Column5" dataDxfId="40"/>
-    <tableColumn id="6" xr3:uid="{F13EA15F-52B4-418E-8DAC-62EF7C15F12C}" name="Column6" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{15D4A987-6071-4E92-9B4E-8D02D281010E}" name="Column7" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{86C689AB-35C1-47AA-98DD-C9CAE4190F81}" name="Column8" dataDxfId="37"/>
-    <tableColumn id="9" xr3:uid="{330B2934-721F-4FA0-B3DF-7050F85C8485}" name="Column9" dataDxfId="36"/>
-    <tableColumn id="10" xr3:uid="{5A571DCC-C03F-475A-952C-9BAE0484FC34}" name="Column10" dataDxfId="35"/>
-    <tableColumn id="11" xr3:uid="{5AC11DCC-9AB8-47E7-8708-E30B1A50C2CA}" name="Column11" dataDxfId="34"/>
-    <tableColumn id="12" xr3:uid="{DABD9820-23AD-407C-9E8B-8B8BA56C1D12}" name="Column12" dataDxfId="33"/>
-    <tableColumn id="13" xr3:uid="{A2448660-9B37-408C-AA88-DED1E04C686C}" name="Column13" dataDxfId="32"/>
-    <tableColumn id="14" xr3:uid="{3CC263F0-E53C-4C42-8BDF-84BF3AE5C037}" name="Column14" dataDxfId="31"/>
-    <tableColumn id="15" xr3:uid="{EB2D926F-B6AA-4F0D-B4B7-CD6799E9615E}" name="Column15" dataDxfId="30"/>
-    <tableColumn id="16" xr3:uid="{4C293917-C86B-4B10-856C-81D5D98BEFBD}" name="Column16" dataDxfId="29"/>
-    <tableColumn id="17" xr3:uid="{ED396F5F-4827-4878-8F96-197FACF57EAA}" name="Column17" dataDxfId="28"/>
-    <tableColumn id="18" xr3:uid="{29D55304-C60A-4F11-BE0D-4726EF5B3BFE}" name="Column18" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{F80A0028-6831-49DC-A737-1843B2BDFB25}" name="Column3" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{B38F8820-4A19-4584-B056-E19957264855}" name="Column4" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{3356337E-64E9-4C20-A5B2-665734CA49EE}" name="Column5" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{F13EA15F-52B4-418E-8DAC-62EF7C15F12C}" name="Column6" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{15D4A987-6071-4E92-9B4E-8D02D281010E}" name="Column7" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{86C689AB-35C1-47AA-98DD-C9CAE4190F81}" name="Column8" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{330B2934-721F-4FA0-B3DF-7050F85C8485}" name="Column9" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{5A571DCC-C03F-475A-952C-9BAE0484FC34}" name="Column10" dataDxfId="16"/>
+    <tableColumn id="11" xr3:uid="{5AC11DCC-9AB8-47E7-8708-E30B1A50C2CA}" name="Column11" dataDxfId="15"/>
+    <tableColumn id="12" xr3:uid="{DABD9820-23AD-407C-9E8B-8B8BA56C1D12}" name="Column12" dataDxfId="14"/>
+    <tableColumn id="13" xr3:uid="{A2448660-9B37-408C-AA88-DED1E04C686C}" name="Column13" dataDxfId="13"/>
+    <tableColumn id="14" xr3:uid="{3CC263F0-E53C-4C42-8BDF-84BF3AE5C037}" name="Column14" dataDxfId="12"/>
+    <tableColumn id="15" xr3:uid="{EB2D926F-B6AA-4F0D-B4B7-CD6799E9615E}" name="Column15" dataDxfId="11"/>
+    <tableColumn id="16" xr3:uid="{4C293917-C86B-4B10-856C-81D5D98BEFBD}" name="Column16" dataDxfId="10"/>
+    <tableColumn id="17" xr3:uid="{ED396F5F-4827-4878-8F96-197FACF57EAA}" name="Column17" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{29D55304-C60A-4F11-BE0D-4726EF5B3BFE}" name="Column18" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC50A23E-B3D4-4C8D-830A-200F854F0A55}" name="Table1" displayName="Table1" ref="A2:C9" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC50A23E-B3D4-4C8D-830A-200F854F0A55}" name="Table1" displayName="Table1" ref="A2:C9" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A2:C9" xr:uid="{FC50A23E-B3D4-4C8D-830A-200F854F0A55}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{1BCBBE5C-F7E0-4EEF-80FA-13F53AE44EAE}" name="TC" dataDxfId="24" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{BE337629-75A8-42D2-AD2C-1CBB2FFC92AF}" name="Đường đi" dataDxfId="23" dataCellStyle="Normal"/>
-    <tableColumn id="3" xr3:uid="{EE5679A3-3696-4E8E-80D1-CF75CB7F8C4F}" name="Bcov" dataDxfId="22" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{1BCBBE5C-F7E0-4EEF-80FA-13F53AE44EAE}" name="TC" dataDxfId="49" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{BE337629-75A8-42D2-AD2C-1CBB2FFC92AF}" name="Đường đi" dataDxfId="48" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{EE5679A3-3696-4E8E-80D1-CF75CB7F8C4F}" name="Bcov" dataDxfId="47" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0A27A8C5-3F79-4A94-80F3-D155DBE02E1C}" name="Table4" displayName="Table4" ref="A12:G19" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0A27A8C5-3F79-4A94-80F3-D155DBE02E1C}" name="Table4" displayName="Table4" ref="A12:G19" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
   <autoFilter ref="A12:G19" xr:uid="{0A27A8C5-3F79-4A94-80F3-D155DBE02E1C}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6CCBA654-60F8-4191-8627-F30B983C9F98}" name="TC" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{47C6CCED-3BA5-4845-A920-6568AD1FE1C0}" name="loaiGoi" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{D587340E-E827-4CDC-9351-2C316683D5E3}" name="soThang" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{08F0789D-5858-4B4E-9D28-A00C888112F3}" name="doTuoi" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{01E319CD-323B-4045-BC52-87F6F8C19FCF}" name="coSinhVien" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{A7C355DF-97D9-4723-8199-0ABE11070E97}" name="Expected Output" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{581C8684-A2AD-4475-AA14-874BD9A6C7A2}" name="Result" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{6CCBA654-60F8-4191-8627-F30B983C9F98}" name="TC" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{47C6CCED-3BA5-4845-A920-6568AD1FE1C0}" name="loaiGoi" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{D587340E-E827-4CDC-9351-2C316683D5E3}" name="soThang" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{08F0789D-5858-4B4E-9D28-A00C888112F3}" name="doTuoi" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{01E319CD-323B-4045-BC52-87F6F8C19FCF}" name="coSinhVien" dataDxfId="40"/>
+    <tableColumn id="6" xr3:uid="{A7C355DF-97D9-4723-8199-0ABE11070E97}" name="Expected Output" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{581C8684-A2AD-4475-AA14-874BD9A6C7A2}" name="Result" dataDxfId="38"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{79C550E2-0F27-41A3-A2BB-76BAF38CD421}" name="Table26" displayName="Table26" ref="A1:F16" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="A1:F16" xr:uid="{E66FDF7E-B7E6-4FD3-80B9-011B00FC313C}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{07227548-E176-45D1-939A-15D1D090AC24}" name="DU-pair" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{4A16FDA1-420E-45C8-895B-30F6AAE77855}" name="Def-clear path" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{0DC2AC1F-C84C-4965-BCBE-0C1B0C69D70F}" name="Complete path" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{6A9ED1E4-277B-4628-9913-8311A7A2ADB5}" name="Test case (loaiGoi, soThang, doTuoi, coSV)" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{FB1B8230-B9A0-461B-9F6C-5858642426D2}" name="Expected Output" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{6FFEFAEC-EFC2-48DA-BC1C-D6180FF6643B}" name="Result" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3631,12 +3939,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="10"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -3727,15 +4035,15 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
@@ -3779,7 +4087,7 @@
       <c r="F13" s="7">
         <v>-1</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="10" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3802,7 +4110,7 @@
       <c r="F14" s="7">
         <v>-1</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="10" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3825,7 +4133,7 @@
       <c r="F15" s="7">
         <v>-1</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="10" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3848,7 +4156,7 @@
       <c r="F16" s="7">
         <v>-1</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="10" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3871,7 +4179,7 @@
       <c r="F17" s="8">
         <v>540</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" s="10" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3894,7 +4202,7 @@
       <c r="F18" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="10" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3917,7 +4225,7 @@
       <c r="F19" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="10" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3932,4 +4240,343 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E730CC6-0118-46FF-8A88-B8CA7D4FBB08}">
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.19921875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E2" s="7">
+        <v>-1</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="E3" s="7">
+        <v>-1</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="E4" s="7">
+        <v>-1</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="E5" s="7">
+        <v>-1</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E6" s="7">
+        <v>300000</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E7" s="7">
+        <v>300000</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="E8" s="7">
+        <v>1900000</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="E9" s="7">
+        <v>2295000</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="E10" s="7">
+        <v>1377000</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E11" s="7">
+        <v>900000</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="E12" s="7">
+        <v>1530000</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" s="7">
+        <v>1530000</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="E14" s="7">
+        <v>1300000</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="E15" s="7">
+        <v>1377000</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="E16" s="7">
+        <v>1377000</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>